<commit_message>
Middle East inventories correction
</commit_message>
<xml_diff>
--- a/Results/GWP 20a/ammonia climate change GWP 20a results.xlsx
+++ b/Results/GWP 20a/ammonia climate change GWP 20a results.xlsx
@@ -798,7 +798,7 @@
         <v>0.8466439318651791</v>
       </c>
       <c r="N4" t="n">
-        <v>8.577289212489287</v>
+        <v>0.6283920753388644</v>
       </c>
       <c r="O4" t="n">
         <v>0.6102474429785583</v>
@@ -974,7 +974,7 @@
         <v>0.9872398089887113</v>
       </c>
       <c r="N6" t="n">
-        <v>8.577289212489287</v>
+        <v>0.6603263987140341</v>
       </c>
       <c r="O6" t="n">
         <v>0.6421816480633417</v>
@@ -1062,7 +1062,7 @@
         <v>0.9803011900076839</v>
       </c>
       <c r="N7" t="n">
-        <v>8.577289212489287</v>
+        <v>0.7620493334813696</v>
       </c>
       <c r="O7" t="n">
         <v>0.7435207789030881</v>
@@ -1150,7 +1150,7 @@
         <v>1.194292094088296</v>
       </c>
       <c r="N8" t="n">
-        <v>8.577289212489287</v>
+        <v>0.8573143022612257</v>
       </c>
       <c r="O8" t="n">
         <v>0.8717965877469442</v>
@@ -1238,7 +1238,7 @@
         <v>1.556970010411926</v>
       </c>
       <c r="N9" t="n">
-        <v>8.577289212489287</v>
+        <v>1.33871815388561</v>
       </c>
       <c r="O9" t="n">
         <v>1.374914441679641</v>
@@ -1634,7 +1634,7 @@
         <v>0.1428889821975032</v>
       </c>
       <c r="F4" t="n">
-        <v>0.02379443171244244</v>
+        <v>0.02379443171244246</v>
       </c>
       <c r="G4" t="n">
         <v>0.2212339638749498</v>
@@ -1658,7 +1658,7 @@
         <v>0.1328967606241638</v>
       </c>
       <c r="N4" t="n">
-        <v>0.108898240801468</v>
+        <v>0.1501235304984708</v>
       </c>
       <c r="O4" t="n">
         <v>0.06013604520329613</v>
@@ -1670,7 +1670,7 @@
         <v>0.1656099386507632</v>
       </c>
       <c r="R4" t="n">
-        <v>-0.2180095404541156</v>
+        <v>-0.2180095404541155</v>
       </c>
       <c r="S4" t="n">
         <v>0.04909239398504364</v>
@@ -1834,7 +1834,7 @@
         <v>0.1459026411760664</v>
       </c>
       <c r="N6" t="n">
-        <v>0.108898240801468</v>
+        <v>0.1634898595958399</v>
       </c>
       <c r="O6" t="n">
         <v>0.1241720399831645</v>
@@ -1922,7 +1922,7 @@
         <v>0.2111055461444566</v>
       </c>
       <c r="N7" t="n">
-        <v>0.108898240801468</v>
+        <v>0.2283323160187646</v>
       </c>
       <c r="O7" t="n">
         <v>0.1380113791397697</v>
@@ -2010,7 +2010,7 @@
         <v>0.3047407955703738</v>
       </c>
       <c r="N8" t="n">
-        <v>0.108898240801468</v>
+        <v>0.2631849016475273</v>
       </c>
       <c r="O8" t="n">
         <v>0.189351402763602</v>
@@ -2098,7 +2098,7 @@
         <v>0.4189890071493913</v>
       </c>
       <c r="N9" t="n">
-        <v>0.108898240801468</v>
+        <v>0.4362157770236998</v>
       </c>
       <c r="O9" t="n">
         <v>0.3684436648600062</v>
@@ -2518,7 +2518,7 @@
         <v>0.7865872689118614</v>
       </c>
       <c r="N4" t="n">
-        <v>6.961714305217533</v>
+        <v>0.5572323305931769</v>
       </c>
       <c r="O4" t="n">
         <v>0.5348917863329984</v>
@@ -2694,7 +2694,7 @@
         <v>0.9101862707871602</v>
       </c>
       <c r="N6" t="n">
-        <v>6.961714305217533</v>
+        <v>0.5834830909269865</v>
       </c>
       <c r="O6" t="n">
         <v>0.5612657202870994</v>
@@ -2782,7 +2782,7 @@
         <v>0.9057519833504183</v>
       </c>
       <c r="N7" t="n">
-        <v>6.961714305217533</v>
+        <v>0.6763970450317341</v>
       </c>
       <c r="O7" t="n">
         <v>0.6536974897877964</v>
@@ -2870,7 +2870,7 @@
         <v>1.094934650516382</v>
       </c>
       <c r="N8" t="n">
-        <v>6.961714305217533</v>
+        <v>0.7602569846510007</v>
       </c>
       <c r="O8" t="n">
         <v>0.7668600403769219</v>
@@ -2958,7 +2958,7 @@
         <v>1.360975622033845</v>
       </c>
       <c r="N9" t="n">
-        <v>6.961714305217533</v>
+        <v>1.13162068371516</v>
       </c>
       <c r="O9" t="n">
         <v>1.153487900991823</v>
@@ -3166,85 +3166,85 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>2.993704286083266</v>
+        <v>2.993704286083269</v>
       </c>
       <c r="C2" t="n">
-        <v>2.973179169266134</v>
+        <v>2.973179169266136</v>
       </c>
       <c r="D2" t="n">
         <v>3.006090059820969</v>
       </c>
       <c r="E2" t="n">
-        <v>2.983401361808401</v>
+        <v>2.983401361808403</v>
       </c>
       <c r="F2" t="n">
-        <v>2.984673760201456</v>
+        <v>2.984673760201459</v>
       </c>
       <c r="G2" t="n">
-        <v>3.023249526712759</v>
+        <v>3.023249526712761</v>
       </c>
       <c r="H2" t="n">
-        <v>2.999988632796625</v>
+        <v>2.999988632796627</v>
       </c>
       <c r="I2" t="n">
-        <v>2.989338709809477</v>
+        <v>2.98933870980948</v>
       </c>
       <c r="J2" t="n">
-        <v>3.007401118271578</v>
+        <v>3.007401118271581</v>
       </c>
       <c r="K2" t="n">
-        <v>2.994727074639386</v>
+        <v>2.994727074639388</v>
       </c>
       <c r="L2" t="n">
-        <v>3.008779293605888</v>
+        <v>3.008779293605891</v>
       </c>
       <c r="M2" t="n">
-        <v>3.016405375863915</v>
+        <v>3.016405375863917</v>
       </c>
       <c r="N2" t="n">
-        <v>2.995262703401123</v>
+        <v>2.995262703401124</v>
       </c>
       <c r="O2" t="n">
-        <v>3.377887207515207</v>
+        <v>3.377887207515208</v>
       </c>
       <c r="P2" t="n">
-        <v>3.004223319467502</v>
+        <v>3.004223319467503</v>
       </c>
       <c r="Q2" t="n">
         <v>2.982912892594884</v>
       </c>
       <c r="R2" t="n">
-        <v>2.995013857550892</v>
+        <v>2.995013857550895</v>
       </c>
       <c r="S2" t="n">
-        <v>3.007133908903144</v>
+        <v>3.007133908903147</v>
       </c>
       <c r="T2" t="n">
-        <v>2.993365681091113</v>
+        <v>2.993365681091114</v>
       </c>
       <c r="U2" t="n">
-        <v>3.771206933615795</v>
+        <v>3.771206933615797</v>
       </c>
       <c r="V2" t="n">
-        <v>2.988724585304755</v>
+        <v>2.988724585304758</v>
       </c>
       <c r="W2" t="n">
         <v>3.776961558344381</v>
       </c>
       <c r="X2" t="n">
-        <v>3.011137766632613</v>
+        <v>3.011137766632617</v>
       </c>
       <c r="Y2" t="n">
-        <v>3.007283865400357</v>
+        <v>3.007283865400359</v>
       </c>
       <c r="Z2" t="n">
-        <v>3.274753792457812</v>
+        <v>3.274753792457815</v>
       </c>
       <c r="AA2" t="n">
-        <v>3.002261503898954</v>
+        <v>3.002261503898956</v>
       </c>
       <c r="AB2" t="n">
-        <v>3.018371321593318</v>
+        <v>3.018371321593319</v>
       </c>
     </row>
     <row r="3">
@@ -3257,7 +3257,7 @@
         <v>2.169998832300358</v>
       </c>
       <c r="C3" t="n">
-        <v>2.081593485156299</v>
+        <v>2.0815934851563</v>
       </c>
       <c r="D3" t="n">
         <v>2.259541761117164</v>
@@ -3266,19 +3266,19 @@
         <v>2.096990469535405</v>
       </c>
       <c r="F3" t="n">
-        <v>2.106311819476156</v>
+        <v>2.106311819476155</v>
       </c>
       <c r="G3" t="n">
-        <v>2.380000594206514</v>
+        <v>2.380000594206515</v>
       </c>
       <c r="H3" t="n">
-        <v>2.216530223456968</v>
+        <v>2.216530223456967</v>
       </c>
       <c r="I3" t="n">
         <v>2.139816015726281</v>
       </c>
       <c r="J3" t="n">
-        <v>2.267829096518155</v>
+        <v>2.267829096518154</v>
       </c>
       <c r="K3" t="n">
         <v>2.177295770275555</v>
@@ -3290,13 +3290,13 @@
         <v>2.337229054823425</v>
       </c>
       <c r="N3" t="n">
-        <v>2.181889060175932</v>
+        <v>2.181889060175931</v>
       </c>
       <c r="O3" t="n">
         <v>2.810682699147954</v>
       </c>
       <c r="P3" t="n">
-        <v>2.244716122716509</v>
+        <v>2.24471612271651</v>
       </c>
       <c r="Q3" t="n">
         <v>2.093549620553586</v>
@@ -3311,22 +3311,22 @@
         <v>2.168593378195403</v>
       </c>
       <c r="U3" t="n">
-        <v>3.508189835317334</v>
+        <v>3.508189835317335</v>
       </c>
       <c r="V3" t="n">
         <v>2.134303397715203</v>
       </c>
       <c r="W3" t="n">
-        <v>3.581154663459959</v>
+        <v>3.581154663459956</v>
       </c>
       <c r="X3" t="n">
         <v>2.295433344627467</v>
       </c>
       <c r="Y3" t="n">
-        <v>2.267416003160079</v>
+        <v>2.26741600316008</v>
       </c>
       <c r="Z3" t="n">
-        <v>2.642309239816913</v>
+        <v>2.642309239816914</v>
       </c>
       <c r="AA3" t="n">
         <v>2.231678926194728</v>
@@ -3342,85 +3342,85 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.4509364288023366</v>
+        <v>0.4509364288023376</v>
       </c>
       <c r="C4" t="n">
-        <v>0.3373374968763544</v>
+        <v>0.3373374968763546</v>
       </c>
       <c r="D4" t="n">
-        <v>0.5908394409071062</v>
+        <v>0.5908394409071066</v>
       </c>
       <c r="E4" t="n">
-        <v>0.3345601595384415</v>
+        <v>0.334560159538442</v>
       </c>
       <c r="F4" t="n">
-        <v>0.3489324847201433</v>
+        <v>0.3489324847201439</v>
       </c>
       <c r="G4" t="n">
-        <v>0.7846635131946685</v>
+        <v>0.7846635131946695</v>
       </c>
       <c r="H4" t="n">
-        <v>0.5219210158720616</v>
+        <v>0.521921015872062</v>
       </c>
       <c r="I4" t="n">
-        <v>0.4016252365256062</v>
+        <v>0.401625236525607</v>
       </c>
       <c r="J4" t="n">
-        <v>0.605243717358375</v>
+        <v>0.6052437173583749</v>
       </c>
       <c r="K4" t="n">
-        <v>0.462489296049708</v>
+        <v>0.4624892960497082</v>
       </c>
       <c r="L4" t="n">
-        <v>0.6212155736164425</v>
+        <v>0.6212155736164413</v>
       </c>
       <c r="M4" t="n">
-        <v>0.7138525939991159</v>
+        <v>0.7138525939991175</v>
       </c>
       <c r="N4" t="n">
-        <v>5.042007288042453</v>
+        <v>0.4685394693149096</v>
       </c>
       <c r="O4" t="n">
-        <v>0.465285801164692</v>
+        <v>0.4652858011646928</v>
       </c>
       <c r="P4" t="n">
-        <v>0.5697537498717062</v>
+        <v>0.5697537498717069</v>
       </c>
       <c r="Q4" t="n">
-        <v>0.3290426750647912</v>
+        <v>0.3290426750647917</v>
       </c>
       <c r="R4" t="n">
-        <v>0.4657286409618305</v>
+        <v>0.4657286409618304</v>
       </c>
       <c r="S4" t="n">
-        <v>0.6026301964845736</v>
+        <v>0.6026301964845742</v>
       </c>
       <c r="T4" t="n">
-        <v>0.4471117296499826</v>
+        <v>0.4471117296499839</v>
       </c>
       <c r="U4" t="n">
-        <v>0.5591491323338141</v>
+        <v>0.559149132333816</v>
       </c>
       <c r="V4" t="n">
-        <v>0.3919713724837046</v>
+        <v>0.3919713724837041</v>
       </c>
       <c r="W4" t="n">
-        <v>0.6931089649941781</v>
+        <v>0.6931089649941783</v>
       </c>
       <c r="X4" t="n">
-        <v>0.6478556114045044</v>
+        <v>0.6478556114045048</v>
       </c>
       <c r="Y4" t="n">
-        <v>0.6001019606881984</v>
+        <v>0.6001019606881994</v>
       </c>
       <c r="Z4" t="n">
-        <v>0.4691309144170134</v>
+        <v>0.4691309144170138</v>
       </c>
       <c r="AA4" t="n">
-        <v>0.5475941405452373</v>
+        <v>0.5475941405452376</v>
       </c>
       <c r="AB4" t="n">
-        <v>0.727322293227378</v>
+        <v>0.7273222932273783</v>
       </c>
     </row>
     <row r="5">
@@ -3430,13 +3430,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4.332814020114644</v>
+        <v>4.332814020114633</v>
       </c>
       <c r="C5" t="n">
-        <v>2.579399721993859</v>
+        <v>2.579399721993858</v>
       </c>
       <c r="D5" t="n">
-        <v>7.400619806973491</v>
+        <v>7.400619806973489</v>
       </c>
       <c r="E5" t="n">
         <v>2.546120308779971</v>
@@ -3445,70 +3445,70 @@
         <v>2.924785372985711</v>
       </c>
       <c r="G5" t="n">
-        <v>9.787533700492958</v>
+        <v>9.787533700492972</v>
       </c>
       <c r="H5" t="n">
-        <v>6.45875317168948</v>
+        <v>6.458753171689494</v>
       </c>
       <c r="I5" t="n">
-        <v>3.965683970538863</v>
+        <v>3.965683970538861</v>
       </c>
       <c r="J5" t="n">
-        <v>7.107763839782042</v>
+        <v>7.107763839782036</v>
       </c>
       <c r="K5" t="n">
-        <v>4.535717864343332</v>
+        <v>4.535717864343331</v>
       </c>
       <c r="L5" t="n">
-        <v>7.555647460900432</v>
+        <v>7.555647460900408</v>
       </c>
       <c r="M5" t="n">
-        <v>9.854320195075708</v>
+        <v>9.854320195075687</v>
       </c>
       <c r="N5" t="n">
-        <v>5.042007288042453</v>
+        <v>5.042007288042454</v>
       </c>
       <c r="O5" t="n">
-        <v>4.35336735602296</v>
+        <v>4.353367356022974</v>
       </c>
       <c r="P5" t="n">
-        <v>6.248990092951697</v>
+        <v>6.24899009295171</v>
       </c>
       <c r="Q5" t="n">
         <v>2.472051602951899</v>
       </c>
       <c r="R5" t="n">
-        <v>5.259878468570383</v>
+        <v>5.259878468570382</v>
       </c>
       <c r="S5" t="n">
-        <v>6.864649284462942</v>
+        <v>6.864649284462947</v>
       </c>
       <c r="T5" t="n">
-        <v>4.789189756598449</v>
+        <v>4.789189756598447</v>
       </c>
       <c r="U5" t="n">
-        <v>6.364637505375476</v>
+        <v>6.364637505375523</v>
       </c>
       <c r="V5" t="n">
-        <v>3.254901189405972</v>
+        <v>3.254901189405979</v>
       </c>
       <c r="W5" t="n">
-        <v>8.937148475699351</v>
+        <v>8.937148475699336</v>
       </c>
       <c r="X5" t="n">
-        <v>8.339524174632748</v>
+        <v>8.33952417463278</v>
       </c>
       <c r="Y5" t="n">
         <v>7.304339681036744</v>
       </c>
       <c r="Z5" t="n">
-        <v>4.421113475410813</v>
+        <v>4.421113475410801</v>
       </c>
       <c r="AA5" t="n">
-        <v>6.356825827897234</v>
+        <v>6.35682582789723</v>
       </c>
       <c r="AB5" t="n">
-        <v>10.50851130629887</v>
+        <v>10.50851130629886</v>
       </c>
     </row>
     <row r="6">
@@ -3521,61 +3521,61 @@
         <v>0.5629905267805632</v>
       </c>
       <c r="C6" t="n">
-        <v>0.3623137050668395</v>
+        <v>0.3623137050668393</v>
       </c>
       <c r="D6" t="n">
-        <v>0.7028935388853327</v>
+        <v>0.7028935388853328</v>
       </c>
       <c r="E6" t="n">
-        <v>0.446614257516668</v>
+        <v>0.4466142575166678</v>
       </c>
       <c r="F6" t="n">
-        <v>0.3739086929106279</v>
+        <v>0.3739086929106282</v>
       </c>
       <c r="G6" t="n">
-        <v>0.8096397213851523</v>
+        <v>0.8096397213851533</v>
       </c>
       <c r="H6" t="n">
-        <v>0.5468972240625467</v>
+        <v>0.5468972240625473</v>
       </c>
       <c r="I6" t="n">
-        <v>0.4266014447160909</v>
+        <v>0.4266014447160911</v>
       </c>
       <c r="J6" t="n">
-        <v>0.7172978153366034</v>
+        <v>0.7172978153366032</v>
       </c>
       <c r="K6" t="n">
-        <v>0.5745433940279348</v>
+        <v>0.5745433940279353</v>
       </c>
       <c r="L6" t="n">
-        <v>0.733269671594669</v>
+        <v>0.7332696715946693</v>
       </c>
       <c r="M6" t="n">
-        <v>0.7388288021896008</v>
+        <v>0.7388288021896006</v>
       </c>
       <c r="N6" t="n">
-        <v>5.042007288042453</v>
+        <v>0.4941668875411535</v>
       </c>
       <c r="O6" t="n">
-        <v>0.5819163674404928</v>
+        <v>0.5819163674404932</v>
       </c>
       <c r="P6" t="n">
-        <v>0.6863431005981419</v>
+        <v>0.6863431005981432</v>
       </c>
       <c r="Q6" t="n">
         <v>0.4410967730430178</v>
       </c>
       <c r="R6" t="n">
-        <v>0.4907048491523151</v>
+        <v>0.490704849152315</v>
       </c>
       <c r="S6" t="n">
-        <v>0.7146842944627999</v>
+        <v>0.7146842944628</v>
       </c>
       <c r="T6" t="n">
-        <v>0.4720879378404673</v>
+        <v>0.472087937840467</v>
       </c>
       <c r="U6" t="n">
-        <v>0.5883474039400954</v>
+        <v>0.5883474039400971</v>
       </c>
       <c r="V6" t="n">
         <v>0.5040254704619306</v>
@@ -3584,19 +3584,19 @@
         <v>0.8097542325629685</v>
       </c>
       <c r="X6" t="n">
-        <v>0.6728318195949902</v>
+        <v>0.6728318195949895</v>
       </c>
       <c r="Y6" t="n">
-        <v>0.6320802423315823</v>
+        <v>0.6320802423315877</v>
       </c>
       <c r="Z6" t="n">
-        <v>0.58118501239524</v>
+        <v>0.5811850123952397</v>
       </c>
       <c r="AA6" t="n">
-        <v>0.659648238523465</v>
+        <v>0.6596482385234649</v>
       </c>
       <c r="AB6" t="n">
-        <v>0.7545546493959411</v>
+        <v>0.7545546493959425</v>
       </c>
     </row>
     <row r="7">
@@ -3606,85 +3606,85 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.5567867902162271</v>
+        <v>0.5567867902162269</v>
       </c>
       <c r="C7" t="n">
-        <v>0.443187858290246</v>
+        <v>0.4431878582902457</v>
       </c>
       <c r="D7" t="n">
-        <v>0.6966898023209972</v>
+        <v>0.6966898023209975</v>
       </c>
       <c r="E7" t="n">
-        <v>0.4404105209523323</v>
+        <v>0.4404105209523331</v>
       </c>
       <c r="F7" t="n">
-        <v>0.4547828461340337</v>
+        <v>0.4547828461340342</v>
       </c>
       <c r="G7" t="n">
-        <v>0.8905138746085586</v>
+        <v>0.890513874608559</v>
       </c>
       <c r="H7" t="n">
-        <v>0.6277713772859529</v>
+        <v>0.6277713772859531</v>
       </c>
       <c r="I7" t="n">
         <v>0.5074755979394983</v>
       </c>
       <c r="J7" t="n">
-        <v>0.711094078772265</v>
+        <v>0.7110940787722659</v>
       </c>
       <c r="K7" t="n">
-        <v>0.5683396574635989</v>
+        <v>0.5683396574635983</v>
       </c>
       <c r="L7" t="n">
-        <v>0.727065935030334</v>
+        <v>0.7270659350303335</v>
       </c>
       <c r="M7" t="n">
-        <v>0.8197029554130058</v>
+        <v>0.8197029554130072</v>
       </c>
       <c r="N7" t="n">
-        <v>5.042007288042453</v>
+        <v>0.5743898307288</v>
       </c>
       <c r="O7" t="n">
-        <v>0.570801923104459</v>
+        <v>0.5708019231044595</v>
       </c>
       <c r="P7" t="n">
-        <v>0.6752698718114741</v>
+        <v>0.6752698718114745</v>
       </c>
       <c r="Q7" t="n">
-        <v>0.4348930364786827</v>
+        <v>0.434893036478683</v>
       </c>
       <c r="R7" t="n">
-        <v>0.571579002375721</v>
+        <v>0.5715790023757207</v>
       </c>
       <c r="S7" t="n">
-        <v>0.7084805578984649</v>
+        <v>0.7084805578984648</v>
       </c>
       <c r="T7" t="n">
-        <v>0.5529620910638725</v>
+        <v>0.5529620910638737</v>
       </c>
       <c r="U7" t="n">
-        <v>0.66877623461359</v>
+        <v>0.6687762346135938</v>
       </c>
       <c r="V7" t="n">
-        <v>0.4978217338975954</v>
+        <v>0.497821733897595</v>
       </c>
       <c r="W7" t="n">
-        <v>0.7989593264080685</v>
+        <v>0.7989593264080683</v>
       </c>
       <c r="X7" t="n">
-        <v>0.753705972818397</v>
+        <v>0.7537059728183974</v>
       </c>
       <c r="Y7" t="n">
-        <v>0.7101743855178857</v>
+        <v>0.7101743855178866</v>
       </c>
       <c r="Z7" t="n">
-        <v>0.574981275830904</v>
+        <v>0.5749812758309037</v>
       </c>
       <c r="AA7" t="n">
-        <v>0.6534445019591294</v>
+        <v>0.6534445019591297</v>
       </c>
       <c r="AB7" t="n">
-        <v>0.8331726546412703</v>
+        <v>0.8331726546412717</v>
       </c>
     </row>
     <row r="8">
@@ -3694,85 +3694,85 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.6021482462641843</v>
+        <v>0.6021482462641856</v>
       </c>
       <c r="C8" t="n">
-        <v>0.6073554587962872</v>
+        <v>0.6073554587962879</v>
       </c>
       <c r="D8" t="n">
-        <v>0.8608574028270388</v>
+        <v>0.8608574028270395</v>
       </c>
       <c r="E8" t="n">
-        <v>0.5413173541093448</v>
+        <v>0.5413173541093443</v>
       </c>
       <c r="F8" t="n">
-        <v>0.518652910964099</v>
+        <v>0.5186529109640996</v>
       </c>
       <c r="G8" t="n">
         <v>1.079316703113194</v>
       </c>
       <c r="H8" t="n">
-        <v>0.7919389777919965</v>
+        <v>0.7919389777919975</v>
       </c>
       <c r="I8" t="n">
-        <v>0.6716431984455398</v>
+        <v>0.6716431984455402</v>
       </c>
       <c r="J8" t="n">
-        <v>0.8752616792783079</v>
+        <v>0.8752616792783077</v>
       </c>
       <c r="K8" t="n">
-        <v>0.7325072579696414</v>
+        <v>0.7325072579696413</v>
       </c>
       <c r="L8" t="n">
-        <v>0.8912335355363772</v>
+        <v>0.8912335355363769</v>
       </c>
       <c r="M8" t="n">
-        <v>0.9838705559192396</v>
+        <v>0.9838705559192401</v>
       </c>
       <c r="N8" t="n">
-        <v>5.042007288042453</v>
+        <v>0.6464627934278472</v>
       </c>
       <c r="O8" t="n">
-        <v>0.6685175313578291</v>
+        <v>0.66851753135783</v>
       </c>
       <c r="P8" t="n">
-        <v>0.7667817782012145</v>
+        <v>0.7667817782012157</v>
       </c>
       <c r="Q8" t="n">
-        <v>0.4569063735399668</v>
+        <v>0.4569063735399677</v>
       </c>
       <c r="R8" t="n">
-        <v>0.7357466028817643</v>
+        <v>0.7357466028817637</v>
       </c>
       <c r="S8" t="n">
-        <v>0.8726481584045076</v>
+        <v>0.8726481584045087</v>
       </c>
       <c r="T8" t="n">
-        <v>0.7171296915699149</v>
+        <v>0.7171296915699159</v>
       </c>
       <c r="U8" t="n">
-        <v>0.7753153775516823</v>
+        <v>0.7753153775516818</v>
       </c>
       <c r="V8" t="n">
-        <v>0.629422872641899</v>
+        <v>0.6294228726419003</v>
       </c>
       <c r="W8" t="n">
-        <v>0.9631502756606037</v>
+        <v>0.9631502756606044</v>
       </c>
       <c r="X8" t="n">
-        <v>0.7866081290508019</v>
+        <v>0.7866081290508046</v>
       </c>
       <c r="Y8" t="n">
-        <v>0.9923209620152492</v>
+        <v>0.9923209620152502</v>
       </c>
       <c r="Z8" t="n">
-        <v>0.6181358467558297</v>
+        <v>0.6181358467558294</v>
       </c>
       <c r="AA8" t="n">
-        <v>0.8176121024651729</v>
+        <v>0.8176121024651725</v>
       </c>
       <c r="AB8" t="n">
-        <v>1.121443207381977</v>
+        <v>1.121443207381978</v>
       </c>
     </row>
     <row r="9">
@@ -3782,64 +3782,64 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.8234742631727019</v>
+        <v>0.8234742631727022</v>
       </c>
       <c r="C9" t="n">
-        <v>0.8227949203173763</v>
+        <v>0.8227949203173766</v>
       </c>
       <c r="D9" t="n">
-        <v>1.076296864348127</v>
+        <v>1.076296864348128</v>
       </c>
       <c r="E9" t="n">
-        <v>0.7939562343431378</v>
+        <v>0.793956234343137</v>
       </c>
       <c r="F9" t="n">
-        <v>0.5740793824900823</v>
+        <v>0.5740793824900817</v>
       </c>
       <c r="G9" t="n">
-        <v>1.270120978146865</v>
+        <v>1.270120978146864</v>
       </c>
       <c r="H9" t="n">
-        <v>1.007378439313085</v>
+        <v>1.007378439313086</v>
       </c>
       <c r="I9" t="n">
-        <v>0.8870826599666303</v>
+        <v>0.88708265996663</v>
       </c>
       <c r="J9" t="n">
-        <v>1.090701140799397</v>
+        <v>1.090701140799398</v>
       </c>
       <c r="K9" t="n">
         <v>0.947946719490729</v>
       </c>
       <c r="L9" t="n">
-        <v>1.106672997057466</v>
+        <v>1.106672997057465</v>
       </c>
       <c r="M9" t="n">
         <v>1.199310017440139</v>
       </c>
       <c r="N9" t="n">
-        <v>5.042007288042453</v>
+        <v>0.9539968927559319</v>
       </c>
       <c r="O9" t="n">
-        <v>0.9881646838360764</v>
+        <v>0.988164683836077</v>
       </c>
       <c r="P9" t="n">
-        <v>1.10077114885361</v>
+        <v>1.100771148853611</v>
       </c>
       <c r="Q9" t="n">
-        <v>0.8145001400169872</v>
+        <v>0.8145001400169876</v>
       </c>
       <c r="R9" t="n">
-        <v>0.9511860644028514</v>
+        <v>0.9511860644028511</v>
       </c>
       <c r="S9" t="n">
         <v>1.088087619925596</v>
       </c>
       <c r="T9" t="n">
-        <v>0.9325691530910052</v>
+        <v>0.9325691530910056</v>
       </c>
       <c r="U9" t="n">
-        <v>1.048828619190631</v>
+        <v>1.048828619190634</v>
       </c>
       <c r="V9" t="n">
         <v>1.007735486866757</v>
@@ -3851,16 +3851,16 @@
         <v>1.133313034845528</v>
       </c>
       <c r="Y9" t="n">
-        <v>1.089781447545017</v>
+        <v>1.089781447545016</v>
       </c>
       <c r="Z9" t="n">
-        <v>0.8865078833336996</v>
+        <v>0.8865078833336982</v>
       </c>
       <c r="AA9" t="n">
-        <v>1.033051563986261</v>
+        <v>1.033051563986262</v>
       </c>
       <c r="AB9" t="n">
-        <v>1.212779716668402</v>
+        <v>1.212779716668403</v>
       </c>
     </row>
   </sheetData>
@@ -4026,7 +4026,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>2.986440352726758</v>
+        <v>2.986440352726757</v>
       </c>
       <c r="C2" t="n">
         <v>2.969373732505465</v>
@@ -4038,7 +4038,7 @@
         <v>2.975170244442945</v>
       </c>
       <c r="F2" t="n">
-        <v>2.981805155986176</v>
+        <v>2.981805155986177</v>
       </c>
       <c r="G2" t="n">
         <v>3.011194357458953</v>
@@ -4050,22 +4050,22 @@
         <v>2.984178388242388</v>
       </c>
       <c r="J2" t="n">
-        <v>2.999101497669393</v>
+        <v>2.999101497669391</v>
       </c>
       <c r="K2" t="n">
-        <v>2.993622247894012</v>
+        <v>2.993622247894013</v>
       </c>
       <c r="L2" t="n">
-        <v>2.998492806051089</v>
+        <v>2.99849280605109</v>
       </c>
       <c r="M2" t="n">
-        <v>3.005102718192138</v>
+        <v>3.005102718192137</v>
       </c>
       <c r="N2" t="n">
         <v>2.987512842067502</v>
       </c>
       <c r="O2" t="n">
-        <v>3.360494244125724</v>
+        <v>3.360494244125723</v>
       </c>
       <c r="P2" t="n">
         <v>2.997599713574871</v>
@@ -4074,19 +4074,19 @@
         <v>2.981222071111544</v>
       </c>
       <c r="R2" t="n">
-        <v>2.987698298529794</v>
+        <v>2.987698298529793</v>
       </c>
       <c r="S2" t="n">
         <v>2.998794177571321</v>
       </c>
       <c r="T2" t="n">
-        <v>2.987089320939499</v>
+        <v>2.987089320939498</v>
       </c>
       <c r="U2" t="n">
-        <v>3.766077453318106</v>
+        <v>3.766077453318105</v>
       </c>
       <c r="V2" t="n">
-        <v>2.992915645544042</v>
+        <v>2.992915645544041</v>
       </c>
       <c r="W2" t="n">
         <v>3.76959153581853</v>
@@ -4095,16 +4095,16 @@
         <v>3.007918090678546</v>
       </c>
       <c r="Y2" t="n">
-        <v>3.015766752852954</v>
+        <v>3.015766752852953</v>
       </c>
       <c r="Z2" t="n">
-        <v>3.264392202083637</v>
+        <v>3.264392202083636</v>
       </c>
       <c r="AA2" t="n">
-        <v>2.998579365828175</v>
+        <v>2.998579365828176</v>
       </c>
       <c r="AB2" t="n">
-        <v>3.009074116475246</v>
+        <v>3.009074116475248</v>
       </c>
     </row>
     <row r="3">
@@ -4120,25 +4120,25 @@
         <v>2.091059540351124</v>
       </c>
       <c r="D3" t="n">
-        <v>2.186616961037769</v>
+        <v>2.186616961037768</v>
       </c>
       <c r="E3" t="n">
-        <v>2.070541942175246</v>
+        <v>2.070541942175245</v>
       </c>
       <c r="F3" t="n">
         <v>2.118268855554074</v>
       </c>
       <c r="G3" t="n">
-        <v>2.326087007078509</v>
+        <v>2.32608700707851</v>
       </c>
       <c r="H3" t="n">
-        <v>2.193986278384092</v>
+        <v>2.193986278384091</v>
       </c>
       <c r="I3" t="n">
-        <v>2.135309285807349</v>
+        <v>2.135309285807348</v>
       </c>
       <c r="J3" t="n">
-        <v>2.240838068265504</v>
+        <v>2.240838068265503</v>
       </c>
       <c r="K3" t="n">
         <v>2.201764617149726</v>
@@ -4150,10 +4150,10 @@
         <v>2.288315226388756</v>
       </c>
       <c r="N3" t="n">
-        <v>2.159022174394509</v>
+        <v>2.159022174394508</v>
       </c>
       <c r="O3" t="n">
-        <v>2.761863756664854</v>
+        <v>2.761863756664853</v>
       </c>
       <c r="P3" t="n">
         <v>2.229577319479455</v>
@@ -4171,28 +4171,28 @@
         <v>2.156226046996115</v>
       </c>
       <c r="U3" t="n">
-        <v>3.517217684207751</v>
+        <v>3.517217684207752</v>
       </c>
       <c r="V3" t="n">
-        <v>2.196178446837498</v>
+        <v>2.196178446837499</v>
       </c>
       <c r="W3" t="n">
-        <v>3.578602913621354</v>
+        <v>3.578602913621355</v>
       </c>
       <c r="X3" t="n">
         <v>2.304428527358727</v>
       </c>
       <c r="Y3" t="n">
-        <v>2.360761512225863</v>
+        <v>2.360761512225861</v>
       </c>
       <c r="Z3" t="n">
-        <v>2.615653209529639</v>
+        <v>2.615653209529638</v>
       </c>
       <c r="AA3" t="n">
         <v>2.237919914080229</v>
       </c>
       <c r="AB3" t="n">
-        <v>2.312994614426423</v>
+        <v>2.312994614426422</v>
       </c>
     </row>
     <row r="4">
@@ -4202,85 +4202,85 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.4250432200556757</v>
+        <v>0.4250432200556756</v>
       </c>
       <c r="C4" t="n">
-        <v>0.3593073473323504</v>
+        <v>0.3593073473323486</v>
       </c>
       <c r="D4" t="n">
-        <v>0.4811126565622166</v>
+        <v>0.4811126565622144</v>
       </c>
       <c r="E4" t="n">
-        <v>0.2977421624840468</v>
+        <v>0.2977421624840453</v>
       </c>
       <c r="F4" t="n">
-        <v>0.3726865405749621</v>
+        <v>0.3726865405749614</v>
       </c>
       <c r="G4" t="n">
-        <v>0.7046510909105933</v>
+        <v>0.7046510909105891</v>
       </c>
       <c r="H4" t="n">
-        <v>0.4911700680425113</v>
+        <v>0.4911700680425107</v>
       </c>
       <c r="I4" t="n">
-        <v>0.3994932906496654</v>
+        <v>0.3994932906496645</v>
       </c>
       <c r="J4" t="n">
-        <v>0.5677478024695082</v>
+        <v>0.5677478024695057</v>
       </c>
       <c r="K4" t="n">
-        <v>0.5061660298048026</v>
+        <v>0.5061660298048012</v>
       </c>
       <c r="L4" t="n">
-        <v>0.5611812247564434</v>
+        <v>0.5611812247564424</v>
       </c>
       <c r="M4" t="n">
-        <v>0.6425532951092416</v>
+        <v>0.6425532951092392</v>
       </c>
       <c r="N4" t="n">
-        <v>4.45754635868574</v>
+        <v>0.4371574805288559</v>
       </c>
       <c r="O4" t="n">
-        <v>0.4127778362074715</v>
+        <v>0.4127778362074711</v>
       </c>
       <c r="P4" t="n">
-        <v>0.5510933343947148</v>
+        <v>0.5510933343947123</v>
       </c>
       <c r="Q4" t="n">
-        <v>0.3661003286836898</v>
+        <v>0.366100328683689</v>
       </c>
       <c r="R4" t="n">
-        <v>0.4392522965846404</v>
+        <v>0.4392522965846406</v>
       </c>
       <c r="S4" t="n">
-        <v>0.5645853547151972</v>
+        <v>0.5645853547151947</v>
       </c>
       <c r="T4" t="n">
-        <v>0.4323736145586958</v>
+        <v>0.4323736145586936</v>
       </c>
       <c r="U4" t="n">
-        <v>0.586063816965613</v>
+        <v>0.5860638169656094</v>
       </c>
       <c r="V4" t="n">
-        <v>0.4961176683090533</v>
+        <v>0.496117668309053</v>
       </c>
       <c r="W4" t="n">
-        <v>0.7021884796077602</v>
+        <v>0.7021884796077604</v>
       </c>
       <c r="X4" t="n">
-        <v>0.6676441504687124</v>
+        <v>0.6676441504687117</v>
       </c>
       <c r="Y4" t="n">
-        <v>0.7526616844822075</v>
+        <v>0.7526616844822066</v>
       </c>
       <c r="Z4" t="n">
-        <v>0.4393233648760667</v>
+        <v>0.4393233648760655</v>
       </c>
       <c r="AA4" t="n">
-        <v>0.5621589572581008</v>
+        <v>0.5621589572581001</v>
       </c>
       <c r="AB4" t="n">
-        <v>0.6785075179904354</v>
+        <v>0.6785075179904358</v>
       </c>
     </row>
     <row r="5">
@@ -4290,85 +4290,85 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>3.769175731394048</v>
+        <v>3.769175731394055</v>
       </c>
       <c r="C5" t="n">
-        <v>2.913240633959896</v>
+        <v>2.91324063395989</v>
       </c>
       <c r="D5" t="n">
-        <v>5.142544113264734</v>
+        <v>5.142544113264703</v>
       </c>
       <c r="E5" t="n">
-        <v>1.789390876241729</v>
+        <v>1.789390876241728</v>
       </c>
       <c r="F5" t="n">
-        <v>3.308317131334378</v>
+        <v>3.30831713133436</v>
       </c>
       <c r="G5" t="n">
-        <v>8.177388402899554</v>
+        <v>8.177388402899538</v>
       </c>
       <c r="H5" t="n">
-        <v>5.846180482013193</v>
+        <v>5.846180482013196</v>
       </c>
       <c r="I5" t="n">
-        <v>3.835584407665222</v>
+        <v>3.835584407665218</v>
       </c>
       <c r="J5" t="n">
-        <v>6.309673170441192</v>
+        <v>6.30967317044118</v>
       </c>
       <c r="K5" t="n">
-        <v>5.23204500874694</v>
+        <v>5.232045008746944</v>
       </c>
       <c r="L5" t="n">
-        <v>6.242813223971427</v>
+        <v>6.242813223971431</v>
       </c>
       <c r="M5" t="n">
-        <v>8.14602593859666</v>
+        <v>8.146025938596653</v>
       </c>
       <c r="N5" t="n">
-        <v>4.45754635868574</v>
+        <v>4.457546358685735</v>
       </c>
       <c r="O5" t="n">
-        <v>3.512811694694004</v>
+        <v>3.512811694693989</v>
       </c>
       <c r="P5" t="n">
-        <v>5.728851118172259</v>
+        <v>5.728851118172227</v>
       </c>
       <c r="Q5" t="n">
-        <v>3.034660487934754</v>
+        <v>3.034660487934745</v>
       </c>
       <c r="R5" t="n">
-        <v>4.723497669474847</v>
+        <v>4.723497669474844</v>
       </c>
       <c r="S5" t="n">
-        <v>6.128215681392876</v>
+        <v>6.128215681392871</v>
       </c>
       <c r="T5" t="n">
         <v>4.490346853792426</v>
       </c>
       <c r="U5" t="n">
-        <v>6.561400555517717</v>
+        <v>6.561400555517725</v>
       </c>
       <c r="V5" t="n">
-        <v>4.807358703839619</v>
+        <v>4.807358703839616</v>
       </c>
       <c r="W5" t="n">
-        <v>9.086666591957977</v>
+        <v>9.086666591957975</v>
       </c>
       <c r="X5" t="n">
-        <v>8.41648603271349</v>
+        <v>8.416486032713467</v>
       </c>
       <c r="Y5" t="n">
-        <v>10.14860016398166</v>
+        <v>10.14860016398165</v>
       </c>
       <c r="Z5" t="n">
-        <v>3.738707681482557</v>
+        <v>3.738707681482556</v>
       </c>
       <c r="AA5" t="n">
-        <v>6.624566038922216</v>
+        <v>6.624566038922211</v>
       </c>
       <c r="AB5" t="n">
-        <v>9.389989312251647</v>
+        <v>9.389989312251625</v>
       </c>
     </row>
     <row r="6">
@@ -4378,85 +4378,85 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.4531872579243933</v>
+        <v>0.4531872579243866</v>
       </c>
       <c r="C6" t="n">
-        <v>0.3874513852010709</v>
+        <v>0.3874513852010605</v>
       </c>
       <c r="D6" t="n">
-        <v>0.5904707456699948</v>
+        <v>0.5904707456699942</v>
       </c>
       <c r="E6" t="n">
-        <v>0.4071002515918251</v>
+        <v>0.4071002515918228</v>
       </c>
       <c r="F6" t="n">
-        <v>0.4008305784436831</v>
+        <v>0.4008305784436723</v>
       </c>
       <c r="G6" t="n">
-        <v>0.7327951287793143</v>
+        <v>0.7327951287793022</v>
       </c>
       <c r="H6" t="n">
-        <v>0.6005281571502895</v>
+        <v>0.6005281571502885</v>
       </c>
       <c r="I6" t="n">
-        <v>0.4276373285183851</v>
+        <v>0.4276373285183744</v>
       </c>
       <c r="J6" t="n">
-        <v>0.6771058915772848</v>
+        <v>0.6771058915772838</v>
       </c>
       <c r="K6" t="n">
-        <v>0.6155241189125804</v>
+        <v>0.6155241189125781</v>
       </c>
       <c r="L6" t="n">
-        <v>0.5893252626251648</v>
+        <v>0.5893252626251551</v>
       </c>
       <c r="M6" t="n">
-        <v>0.6706973329779639</v>
+        <v>0.6706973329779512</v>
       </c>
       <c r="N6" t="n">
-        <v>4.45754635868574</v>
+        <v>0.4664773873887191</v>
       </c>
       <c r="O6" t="n">
-        <v>0.4422102249486296</v>
+        <v>0.4422102249486352</v>
       </c>
       <c r="P6" t="n">
-        <v>0.6653431007327405</v>
+        <v>0.6653431007327389</v>
       </c>
       <c r="Q6" t="n">
-        <v>0.4754584177914669</v>
+        <v>0.4754584177914645</v>
       </c>
       <c r="R6" t="n">
-        <v>0.5486103856924182</v>
+        <v>0.548610385692415</v>
       </c>
       <c r="S6" t="n">
-        <v>0.592729392583913</v>
+        <v>0.5927293925839066</v>
       </c>
       <c r="T6" t="n">
-        <v>0.5417317036664733</v>
+        <v>0.5417317036664717</v>
       </c>
       <c r="U6" t="n">
-        <v>0.6990586218828132</v>
+        <v>0.6990586218828096</v>
       </c>
       <c r="V6" t="n">
-        <v>0.5242617061777719</v>
+        <v>0.5242617061777642</v>
       </c>
       <c r="W6" t="n">
-        <v>0.7357519770785033</v>
+        <v>0.7357519770785029</v>
       </c>
       <c r="X6" t="n">
-        <v>0.6957881883374294</v>
+        <v>0.6957881883374222</v>
       </c>
       <c r="Y6" t="n">
-        <v>0.7881970343333106</v>
+        <v>0.7881970343333009</v>
       </c>
       <c r="Z6" t="n">
-        <v>0.4674674027447873</v>
+        <v>0.4674674027447764</v>
       </c>
       <c r="AA6" t="n">
-        <v>0.6715170463658792</v>
+        <v>0.6715170463658793</v>
       </c>
       <c r="AB6" t="n">
-        <v>0.7088665411384705</v>
+        <v>0.7088665411384709</v>
       </c>
     </row>
     <row r="7">
@@ -4466,85 +4466,85 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.5279621219820432</v>
+        <v>0.5279621219820412</v>
       </c>
       <c r="C7" t="n">
-        <v>0.462226249258717</v>
+        <v>0.462226249258715</v>
       </c>
       <c r="D7" t="n">
-        <v>0.5840315584885839</v>
+        <v>0.5840315584885807</v>
       </c>
       <c r="E7" t="n">
-        <v>0.4006610644104134</v>
+        <v>0.4006610644104114</v>
       </c>
       <c r="F7" t="n">
-        <v>0.47560544250133</v>
+        <v>0.4756054425013264</v>
       </c>
       <c r="G7" t="n">
-        <v>0.8075699928369608</v>
+        <v>0.8075699928369562</v>
       </c>
       <c r="H7" t="n">
-        <v>0.5940889699688789</v>
+        <v>0.5940889699688773</v>
       </c>
       <c r="I7" t="n">
-        <v>0.5024121925760322</v>
+        <v>0.5024121925760305</v>
       </c>
       <c r="J7" t="n">
-        <v>0.6706667043958749</v>
+        <v>0.6706667043958714</v>
       </c>
       <c r="K7" t="n">
-        <v>0.6090849317311692</v>
+        <v>0.6090849317311674</v>
       </c>
       <c r="L7" t="n">
-        <v>0.664100126682812</v>
+        <v>0.6641001266828106</v>
       </c>
       <c r="M7" t="n">
-        <v>0.7454721970356065</v>
+        <v>0.7454721970356037</v>
       </c>
       <c r="N7" t="n">
-        <v>4.45754635868574</v>
+        <v>0.5400763824552197</v>
       </c>
       <c r="O7" t="n">
-        <v>0.515362646109677</v>
+        <v>0.5153626461096744</v>
       </c>
       <c r="P7" t="n">
-        <v>0.6536781442969206</v>
+        <v>0.6536781442969183</v>
       </c>
       <c r="Q7" t="n">
-        <v>0.4690192306100565</v>
+        <v>0.4690192306100555</v>
       </c>
       <c r="R7" t="n">
-        <v>0.5421711985110075</v>
+        <v>0.542171198511007</v>
       </c>
       <c r="S7" t="n">
-        <v>0.6675042566415643</v>
+        <v>0.6675042566415615</v>
       </c>
       <c r="T7" t="n">
-        <v>0.5352925164850637</v>
+        <v>0.5352925164850615</v>
       </c>
       <c r="U7" t="n">
-        <v>0.6918870555450988</v>
+        <v>0.6918870555450977</v>
       </c>
       <c r="V7" t="n">
-        <v>0.5990365702354202</v>
+        <v>0.5990365702354191</v>
       </c>
       <c r="W7" t="n">
-        <v>0.8051073815341271</v>
+        <v>0.8051073815341248</v>
       </c>
       <c r="X7" t="n">
-        <v>0.7705630523950794</v>
+        <v>0.7705630523950781</v>
       </c>
       <c r="Y7" t="n">
-        <v>0.859217302217998</v>
+        <v>0.8592173022179929</v>
       </c>
       <c r="Z7" t="n">
-        <v>0.5422422668024324</v>
+        <v>0.5422422668024315</v>
       </c>
       <c r="AA7" t="n">
-        <v>0.6650778591844676</v>
+        <v>0.6650778591844664</v>
       </c>
       <c r="AB7" t="n">
-        <v>0.7814264199168014</v>
+        <v>0.7814264199168006</v>
       </c>
     </row>
     <row r="8">
@@ -4554,85 +4554,85 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.5695178607506726</v>
+        <v>0.5695178607506722</v>
       </c>
       <c r="C8" t="n">
-        <v>0.6170839634849327</v>
+        <v>0.6170839634849284</v>
       </c>
       <c r="D8" t="n">
-        <v>0.7388892727148002</v>
+        <v>0.7388892727147983</v>
       </c>
       <c r="E8" t="n">
-        <v>0.4951888189151714</v>
+        <v>0.4951888189151689</v>
       </c>
       <c r="F8" t="n">
-        <v>0.5348123048516218</v>
+        <v>0.5348123048516199</v>
       </c>
       <c r="G8" t="n">
-        <v>0.9859216097640291</v>
+        <v>0.9859216097640255</v>
       </c>
       <c r="H8" t="n">
-        <v>0.748946684195094</v>
+        <v>0.7489466841950905</v>
       </c>
       <c r="I8" t="n">
-        <v>0.6572699068022467</v>
+        <v>0.6572699068022442</v>
       </c>
       <c r="J8" t="n">
-        <v>0.8255244186220901</v>
+        <v>0.8255244186220881</v>
       </c>
       <c r="K8" t="n">
-        <v>0.7639426459573848</v>
+        <v>0.7639426459573804</v>
       </c>
       <c r="L8" t="n">
-        <v>0.8189578409090271</v>
+        <v>0.8189578409090233</v>
       </c>
       <c r="M8" t="n">
-        <v>0.9003299112620294</v>
+        <v>0.9003299112620253</v>
       </c>
       <c r="N8" t="n">
-        <v>4.45754635868574</v>
+        <v>0.6071061106801445</v>
       </c>
       <c r="O8" t="n">
-        <v>0.6068623594819506</v>
+        <v>0.606862359481946</v>
       </c>
       <c r="P8" t="n">
-        <v>0.7392615670625347</v>
+        <v>0.7392615670625332</v>
       </c>
       <c r="Q8" t="n">
-        <v>0.4883085452238803</v>
+        <v>0.4883085452238764</v>
       </c>
       <c r="R8" t="n">
-        <v>0.6970289127372227</v>
+        <v>0.6970289127372205</v>
       </c>
       <c r="S8" t="n">
-        <v>0.8223619708677804</v>
+        <v>0.8223619708677773</v>
       </c>
       <c r="T8" t="n">
-        <v>0.6901502307112777</v>
+        <v>0.6901502307112752</v>
       </c>
       <c r="U8" t="n">
-        <v>0.7918673041489833</v>
+        <v>0.7918673041489842</v>
       </c>
       <c r="V8" t="n">
         <v>0.7225867001702155</v>
       </c>
       <c r="W8" t="n">
-        <v>0.959987362791338</v>
+        <v>0.959987362791336</v>
       </c>
       <c r="X8" t="n">
-        <v>0.8002367181612386</v>
+        <v>0.8002367181612352</v>
       </c>
       <c r="Y8" t="n">
-        <v>1.126200559546741</v>
+        <v>1.126200559546737</v>
       </c>
       <c r="Z8" t="n">
-        <v>0.5816933632119319</v>
+        <v>0.5816933632119301</v>
       </c>
       <c r="AA8" t="n">
-        <v>0.8199355734106822</v>
+        <v>0.8199355734106807</v>
       </c>
       <c r="AB8" t="n">
-        <v>1.054637521616486</v>
+        <v>1.054637521616483</v>
       </c>
     </row>
     <row r="9">
@@ -4642,85 +4642,85 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.7638718735692427</v>
+        <v>0.763871873569241</v>
       </c>
       <c r="C9" t="n">
-        <v>0.8012006504656936</v>
+        <v>0.801200650465691</v>
       </c>
       <c r="D9" t="n">
-        <v>0.9230059596955614</v>
+        <v>0.9230059596955574</v>
       </c>
       <c r="E9" t="n">
-        <v>0.7158485857740345</v>
+        <v>0.7158485857740329</v>
       </c>
       <c r="F9" t="n">
-        <v>0.576987661864637</v>
+        <v>0.5769876618646351</v>
       </c>
       <c r="G9" t="n">
-        <v>1.146544421209469</v>
+        <v>1.146544421209466</v>
       </c>
       <c r="H9" t="n">
-        <v>0.9330633711758537</v>
+        <v>0.9330633711758531</v>
       </c>
       <c r="I9" t="n">
-        <v>0.8413865937830095</v>
+        <v>0.8413865937830078</v>
       </c>
       <c r="J9" t="n">
-        <v>1.00964110560285</v>
+        <v>1.009641105602848</v>
       </c>
       <c r="K9" t="n">
-        <v>0.9480593329381443</v>
+        <v>0.9480593329381419</v>
       </c>
       <c r="L9" t="n">
-        <v>1.003074527889788</v>
+        <v>1.003074527889787</v>
       </c>
       <c r="M9" t="n">
-        <v>1.084446598242585</v>
+        <v>1.084446598242581</v>
       </c>
       <c r="N9" t="n">
-        <v>4.45754635868574</v>
+        <v>0.8790507836621957</v>
       </c>
       <c r="O9" t="n">
-        <v>0.8888266654413302</v>
+        <v>0.8888266654413278</v>
       </c>
       <c r="P9" t="n">
-        <v>1.034570398637258</v>
+        <v>1.034570398637255</v>
       </c>
       <c r="Q9" t="n">
-        <v>0.8079936589825666</v>
+        <v>0.8079936589825637</v>
       </c>
       <c r="R9" t="n">
-        <v>0.8811455997179832</v>
+        <v>0.8811455997179809</v>
       </c>
       <c r="S9" t="n">
-        <v>1.006478657848539</v>
+        <v>1.006478657848538</v>
       </c>
       <c r="T9" t="n">
-        <v>0.8742669176920393</v>
+        <v>0.874266917692036</v>
       </c>
       <c r="U9" t="n">
-        <v>1.031593835908379</v>
+        <v>1.031593835908376</v>
       </c>
       <c r="V9" t="n">
-        <v>1.056945292185268</v>
+        <v>1.056945292185266</v>
       </c>
       <c r="W9" t="n">
-        <v>1.144081782741103</v>
+        <v>1.144081782741101</v>
       </c>
       <c r="X9" t="n">
-        <v>1.109537453602055</v>
+        <v>1.109537453602051</v>
       </c>
       <c r="Y9" t="n">
-        <v>1.198191703424975</v>
+        <v>1.198191703424973</v>
       </c>
       <c r="Z9" t="n">
-        <v>0.8190778599420504</v>
+        <v>0.8190778599420477</v>
       </c>
       <c r="AA9" t="n">
-        <v>1.004052260391444</v>
+        <v>1.004052260391441</v>
       </c>
       <c r="AB9" t="n">
-        <v>1.120400821123779</v>
+        <v>1.120400821123778</v>
       </c>
     </row>
   </sheetData>
@@ -5098,7 +5098,7 @@
         <v>0.3317541351051891</v>
       </c>
       <c r="N4" t="n">
-        <v>1.691331155839079</v>
+        <v>0.24222476271739</v>
       </c>
       <c r="O4" t="n">
         <v>0.1990637028952031</v>
@@ -5274,7 +5274,7 @@
         <v>0.4048545964802611</v>
       </c>
       <c r="N6" t="n">
-        <v>1.691331155839079</v>
+        <v>0.2576771052945594</v>
       </c>
       <c r="O6" t="n">
         <v>0.2780606642931328</v>
@@ -5362,7 +5362,7 @@
         <v>0.4220012203806591</v>
       </c>
       <c r="N7" t="n">
-        <v>1.691331155839079</v>
+        <v>0.3324718479928603</v>
       </c>
       <c r="O7" t="n">
         <v>0.2889531872991537</v>
@@ -5450,7 +5450,7 @@
         <v>0.5435517136526616</v>
       </c>
       <c r="N8" t="n">
-        <v>1.691331155839079</v>
+        <v>0.3813758021183459</v>
       </c>
       <c r="O8" t="n">
         <v>0.3581786420147626</v>
@@ -5538,7 +5538,7 @@
         <v>0.7103585909860453</v>
       </c>
       <c r="N9" t="n">
-        <v>1.691331155839079</v>
+        <v>0.6208292185982461</v>
       </c>
       <c r="O9" t="n">
         <v>0.6069618841340646</v>
@@ -5809,7 +5809,7 @@
         <v>2.902685007949389</v>
       </c>
       <c r="W2" t="n">
-        <v>3.65529691153037</v>
+        <v>3.655296911530369</v>
       </c>
       <c r="X2" t="n">
         <v>2.938112210274757</v>
@@ -5958,7 +5958,7 @@
         <v>0.1414742781592483</v>
       </c>
       <c r="N4" t="n">
-        <v>1.527690475611856</v>
+        <v>0.224032542418378</v>
       </c>
       <c r="O4" t="n">
         <v>0.1461283222226495</v>
@@ -6034,7 +6034,7 @@
         <v>0.118516318844847</v>
       </c>
       <c r="J5" t="n">
-        <v>0.8235873217233159</v>
+        <v>0.8235873217233158</v>
       </c>
       <c r="K5" t="n">
         <v>0.01569835881204307</v>
@@ -6064,7 +6064,7 @@
         <v>-0.1693543144540846</v>
       </c>
       <c r="T5" t="n">
-        <v>-0.6619669004124539</v>
+        <v>-0.6619669004124541</v>
       </c>
       <c r="U5" t="n">
         <v>0.5581983248899463</v>
@@ -6119,7 +6119,7 @@
         <v>0.2311486357102975</v>
       </c>
       <c r="I6" t="n">
-        <v>0.1933781674583297</v>
+        <v>0.1933781674583298</v>
       </c>
       <c r="J6" t="n">
         <v>0.2381605766736878</v>
@@ -6134,13 +6134,13 @@
         <v>0.1930415477330304</v>
       </c>
       <c r="N6" t="n">
-        <v>1.527690475611856</v>
+        <v>0.2315830583589296</v>
       </c>
       <c r="O6" t="n">
         <v>0.2027071176766492</v>
       </c>
       <c r="P6" t="n">
-        <v>0.05401769721940876</v>
+        <v>0.05401769721940872</v>
       </c>
       <c r="Q6" t="n">
         <v>0.2093437406994041</v>
@@ -6189,13 +6189,13 @@
         <v>0.1216729149297804</v>
       </c>
       <c r="C7" t="n">
-        <v>0.2481916295323058</v>
+        <v>0.2481916295323057</v>
       </c>
       <c r="D7" t="n">
         <v>0.2536647034336234</v>
       </c>
       <c r="E7" t="n">
-        <v>0.04055109832677881</v>
+        <v>0.04055109832677876</v>
       </c>
       <c r="F7" t="n">
         <v>0.08256434531173819</v>
@@ -6219,16 +6219,16 @@
         <v>0.03997489755752823</v>
       </c>
       <c r="M7" t="n">
-        <v>0.2162913414615454</v>
+        <v>0.2162913414615455</v>
       </c>
       <c r="N7" t="n">
-        <v>1.527690475611856</v>
+        <v>0.2988496057206765</v>
       </c>
       <c r="O7" t="n">
         <v>0.220612274714921</v>
       </c>
       <c r="P7" t="n">
-        <v>0.1225142941901688</v>
+        <v>0.1225142941901689</v>
       </c>
       <c r="Q7" t="n">
         <v>0.2325935344279199</v>
@@ -6274,7 +6274,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.1371800263840397</v>
+        <v>0.1371800263840396</v>
       </c>
       <c r="C8" t="n">
         <v>0.3349918164363931</v>
@@ -6283,7 +6283,7 @@
         <v>0.3404648903377097</v>
       </c>
       <c r="E8" t="n">
-        <v>0.08938982556443745</v>
+        <v>0.08938982556443742</v>
       </c>
       <c r="F8" t="n">
         <v>0.1091780847020447</v>
@@ -6307,10 +6307,10 @@
         <v>0.1267750844616161</v>
       </c>
       <c r="M8" t="n">
-        <v>0.3030915283655542</v>
+        <v>0.3030915283655543</v>
       </c>
       <c r="N8" t="n">
-        <v>1.527690475611856</v>
+        <v>0.3303857320817539</v>
       </c>
       <c r="O8" t="n">
         <v>0.2676685555799957</v>
@@ -6322,7 +6322,7 @@
         <v>0.2340899293665713</v>
       </c>
       <c r="R8" t="n">
-        <v>-0.04649233458684229</v>
+        <v>-0.04649233458684224</v>
       </c>
       <c r="S8" t="n">
         <v>0.2825518299341981</v>
@@ -6331,7 +6331,7 @@
         <v>0.2572300155594371</v>
       </c>
       <c r="U8" t="n">
-        <v>0.2955232504299802</v>
+        <v>0.2955232504299801</v>
       </c>
       <c r="V8" t="n">
         <v>0.3277125465847797</v>
@@ -6395,19 +6395,19 @@
         <v>0.2561050124277415</v>
       </c>
       <c r="M9" t="n">
-        <v>0.4324214563317587</v>
+        <v>0.4324214563317586</v>
       </c>
       <c r="N9" t="n">
-        <v>1.527690475611856</v>
+        <v>0.5149797205908889</v>
       </c>
       <c r="O9" t="n">
         <v>0.4595348605922219</v>
       </c>
       <c r="P9" t="n">
-        <v>0.3663214015271641</v>
+        <v>0.366321401527164</v>
       </c>
       <c r="Q9" t="n">
-        <v>0.4487236678993223</v>
+        <v>0.4487236678993222</v>
       </c>
       <c r="R9" t="n">
         <v>0.08283759337928386</v>
@@ -6818,7 +6818,7 @@
         <v>0.1564721564489442</v>
       </c>
       <c r="N4" t="n">
-        <v>1.795835503947679</v>
+        <v>0.2329230942787951</v>
       </c>
       <c r="O4" t="n">
         <v>0.06829204497842767</v>
@@ -6994,7 +6994,7 @@
         <v>0.2025989484162665</v>
       </c>
       <c r="N6" t="n">
-        <v>1.795835503947679</v>
+        <v>0.2393970495573405</v>
       </c>
       <c r="O6" t="n">
         <v>0.07488006519937355</v>
@@ -7082,7 +7082,7 @@
         <v>0.2281829521606275</v>
       </c>
       <c r="N7" t="n">
-        <v>1.795835503947679</v>
+        <v>0.3046338899904782</v>
       </c>
       <c r="O7" t="n">
         <v>0.1396698927043497</v>
@@ -7170,7 +7170,7 @@
         <v>0.306055067139949</v>
       </c>
       <c r="N8" t="n">
-        <v>1.795835503947679</v>
+        <v>0.3315429282658818</v>
       </c>
       <c r="O8" t="n">
         <v>0.1809169749687997</v>
@@ -7258,7 +7258,7 @@
         <v>0.4195526579477167</v>
       </c>
       <c r="N9" t="n">
-        <v>1.795835503947679</v>
+        <v>0.4960035957775669</v>
       </c>
       <c r="O9" t="n">
         <v>0.3516699058949279</v>
@@ -7678,7 +7678,7 @@
         <v>0.7282308046696757</v>
       </c>
       <c r="N4" t="n">
-        <v>4.709786997503773</v>
+        <v>0.4298793844528412</v>
       </c>
       <c r="O4" t="n">
         <v>0.3879327268849848</v>
@@ -7766,7 +7766,7 @@
         <v>10.06394527642067</v>
       </c>
       <c r="N5" t="n">
-        <v>4.709786997503774</v>
+        <v>4.709786997503773</v>
       </c>
       <c r="O5" t="n">
         <v>3.432157660367561</v>
@@ -7854,7 +7854,7 @@
         <v>0.749688145336339</v>
       </c>
       <c r="N6" t="n">
-        <v>4.709786997503774</v>
+        <v>0.4521286724091398</v>
       </c>
       <c r="O6" t="n">
         <v>0.5053306150209532</v>
@@ -7942,7 +7942,7 @@
         <v>0.8379032537139512</v>
       </c>
       <c r="N7" t="n">
-        <v>4.709786997503774</v>
+        <v>0.5395518334971173</v>
       </c>
       <c r="O7" t="n">
         <v>0.4972465095798479</v>
@@ -8030,7 +8030,7 @@
         <v>1.00534909234617</v>
       </c>
       <c r="N8" t="n">
-        <v>4.709786997503774</v>
+        <v>0.6121225064182438</v>
       </c>
       <c r="O8" t="n">
         <v>0.5962483681372865</v>
@@ -8118,7 +8118,7 @@
         <v>1.262460265374642</v>
       </c>
       <c r="N9" t="n">
-        <v>4.709786997503774</v>
+        <v>0.9641088451578044</v>
       </c>
       <c r="O9" t="n">
         <v>0.9632382586318318</v>
@@ -8538,7 +8538,7 @@
         <v>0.1784437064006704</v>
       </c>
       <c r="N4" t="n">
-        <v>0.7345620924510728</v>
+        <v>0.2014002281762152</v>
       </c>
       <c r="O4" t="n">
         <v>0.1270765482715513</v>
@@ -8714,7 +8714,7 @@
         <v>0.1903884460200657</v>
       </c>
       <c r="N6" t="n">
-        <v>0.7345620924510728</v>
+        <v>0.2139078104301517</v>
       </c>
       <c r="O6" t="n">
         <v>0.2136480682699015</v>
@@ -8802,7 +8802,7 @@
         <v>0.2655482493816264</v>
       </c>
       <c r="N7" t="n">
-        <v>0.7345620924510728</v>
+        <v>0.2885047711571713</v>
       </c>
       <c r="O7" t="n">
         <v>0.2138473416176258</v>
@@ -8890,7 +8890,7 @@
         <v>0.3851891713092128</v>
       </c>
       <c r="N8" t="n">
-        <v>0.7345620924510728</v>
+        <v>0.3371131356454451</v>
       </c>
       <c r="O8" t="n">
         <v>0.2823098192754733</v>
@@ -8978,7 +8978,7 @@
         <v>0.5747011600821709</v>
       </c>
       <c r="N9" t="n">
-        <v>0.7345620924510728</v>
+        <v>0.5976576818577144</v>
       </c>
       <c r="O9" t="n">
         <v>0.553873151142352</v>

</xml_diff>